<commit_message>
Actualizar datos de Cumple.xlsx
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cumple.xlsx
+++ b/Cumple.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,13 +421,16 @@
       <c r="F1" t="str">
         <v>Estado</v>
       </c>
+      <c r="G1" t="str">
+        <v>Foto</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
         <v>20</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" t="str">
         <v>991875140</v>
@@ -439,7 +442,10 @@
         <v>05/01/2000</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -461,6 +467,9 @@
       <c r="F3">
         <v>1</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -481,6 +490,9 @@
       <c r="F4">
         <v>2</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -501,6 +513,9 @@
       <c r="F5">
         <v>2</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -521,6 +536,9 @@
       <c r="F6">
         <v>2</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -541,6 +559,9 @@
       <c r="F7">
         <v>2</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -561,6 +582,9 @@
       <c r="F8">
         <v>2</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -581,6 +605,9 @@
       <c r="F9">
         <v>2</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -601,6 +628,9 @@
       <c r="F10">
         <v>2</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -621,6 +651,9 @@
       <c r="F11">
         <v>2</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -641,6 +674,9 @@
       <c r="F12">
         <v>2</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -661,6 +697,9 @@
       <c r="F13">
         <v>2</v>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -681,6 +720,9 @@
       <c r="F14">
         <v>2</v>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -701,6 +743,9 @@
       <c r="F15">
         <v>2</v>
       </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -721,6 +766,9 @@
       <c r="F16">
         <v>2</v>
       </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -741,6 +789,9 @@
       <c r="F17">
         <v>2</v>
       </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -761,6 +812,9 @@
       <c r="F18">
         <v>2</v>
       </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -781,6 +835,9 @@
       <c r="F19">
         <v>0</v>
       </c>
+      <c r="G19" t="str">
+        <v>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/4gHYSUNDX1BST0ZJTEUAAQEAAAHIAAAAAAQwAABtbnRyUkdCIFhZWiAH4AABAAEAAAAAAABhY3NwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAQAA9tYAAQAAAADTLQAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAlkZXNjAAAA8AAAACRyWFlaAAABFAAAABRnWFlaAAABKAAAABRiWFlaAAABPAAAABR3dHB0AAABUAAAABRyVFJDAAABZAAAAChnVFJDAAABZAAAAChiVFJDAAABZAAAAChjcHJ0AAABjAAAADxtbHVjAAAAAAAAAAEAAAAMZW5VUwAAAAgAAAAcAHMAUgBHAEJYWVogAAAAAAAAb6IAADj1AAADkFhZWiAAAAAAAABimQAAt4UAABjaWFlaIAAAAAAAACSgAAAPhAAAts9YWVogAAAAAAAA9tYAAQAAAADTLXBhcmEAAAAAAAQAAAACZmYAAPKnAAANWQAAE9AAAApbAAAAAAAAAABtbHVjAAAAAAAAAAEAAAAMZW5VUwAAACAAAAAcAEcAbwBvAGcAbABlACAASQBuAGMALgAgADIAMAAxADb/2wBDAAkGBwgHBgkIBwgKCgkLDRYPDQwMDRsUFRAWIB0iIiAdHx8kKDQsJCYxJx8fLT0tMTU3Ojo6Iys/RD84QzQ5Ojf/2wBDAQoKCg0MDRoPDxo3JR8lNzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzc3Nzf/wAARCACgAJ4DASIAAhEBAxEB/8QAHAAAAQUBAQEAAAAAAAAAAAAABQECAwQGAAcI/8QAPBAAAgEDAwEFBQcCBQQDAAAAAQIDAAQRBRIhMQYTQVFhIlJxgZEUMkKhscHRI1MHFUNi8DOC4fEkcpL/xAAaAQACAwEBAAAAAAAAAAAAAAABAwACBAUG/8QAIxEAAgICAgICAwEAAAAAAAAAAAECEQMSITEEE0FRBSIyYf/aAAwDAQACEQMRAD8A9JIpNtThKQx+VbNjHqQ7abip+7Nd3XrU2BqyDFJirPdDxpDEPOpuiaMr4pNtT915Gu7o0d0DVlfbXbfSrIi88UrIi43MBnzNTcOjKm30rttR3msaVYki5vIlYHG0HJz5UJPbnRFnEQLkk43YAA+poewOgZ20m2rNndW19As9s6yRnxHgfI+RqYop8KnsJ6wft9K7Yc9Kv7E8q7CgcCp7Ceso9y3XikETHoKulBXYFT2MOhS7h/Ku7hqunFNPpU3ZNET7qTdTc0mapRYfurt1MzSZqUSx+412TUea7NSiWSZrs1HmuzUolkmax3b6y1i+NsulNsUZDMGxjNa3NDtTvrSCWO3uZxEXUtyDyB5VScnFWhmKKnKmeK9o9Pu9EgaS4PeMx27wQeT8qzC3sjMHMm0qMA+lem9r44r8KoIeFTuB86xVxpsBOyOM7vAKM8VIZbVsbl8Zxf69BHsV21n0nV7dJZWNm7hJVJOMH8Xyr3zdkZzXyve2jW8nANfTOkd6uk2QuM98LdBJn3toz+dMfJnquC9upN1NzTSaFAseWNIWphNJmjRLHFjSbvWm5pM1CE26k3Vne/l99vrSfaJv7j/WrUU3NHupN1Z77TP/AHH/ADrvtU/9x/rQoGxod1duoALq499qUXdx77UaJsHd1duoGLu49808Xk/vUA7BndWb1S70zU7lba7haQqrYRlI246np41dF5N7w+lDtWJNxDeS3CxrGpVlzyw8vhSc6/WzX4k1vVGU1i4hx3FtAscQGAMk/rQWIMpjWNQQH3OSegwR8/hRTUlDe2DnNDtjYJHC+Iz1rKnwdhJdi6Zpv+Z9qbGCQBommV2THBC8n9DXtRNeHW+tS6NqUF1bwLPMCVRGJGc8eHxr1XT9RF/YrLsxuHtKHJwa2QvSzjeU4rM0Giw86bvU/iFCwkWctDn/ALjUiJEG3C3b/tc0bYngvNKg6sPrTe/jzgOpPoar90rBgbeX2uvteuakg01C3EUq5HnxQ2a+A0mPFxEcYcc1G90gztGcHr4VYm0hDjvGKjrguK6WwhKBBu2g5AToPyqjyP6LaIDd0T4LSGJuvsj6VXBvD1xj4VKsd0w5OKbYmh/cn3hXdzn8Ypht58cufrXfZXI5kc/OpZNR/cj367ukH+pSLZZ6kn4mpFsV6bWJoWTUaEj98GlCx++KmWyVf9J/oalSz8ojR2JqV40WRwie0zHAAHWrcmhW02033dnHAHl86uWMCwrvIxI3A9BVllDIwbx4qdkXD4PP+0GmWUN60FqHUBMgk5H/ADisvqERgQIOreFantM93FrJjkVzAHCqSfZ2kZB9PGgN7qVlHPthgN3KgxleEX5+Pypb8aUp0ujdDzoY8VyfIOsdMC//AC7jqPuZ8PWimlalcRzsLJyqLw3kxoXGuq3bN30gEbn2V2gbPhjr860Gm6W6W4FtCzIpAJHiTXVx4444as4OfNLNlc0aDT9YSYrHdqsbn8QPFHFtHYArGSDyCDQOK1g0+NUkSOa9kXIVxlUXzNW9O1EWkwE8zNEx9odAnqAOg9Ky5cafMDViyNcTCy2R8Ym//Y/irEdinQh1P/3FWwmQCHyPMNnNKAw6N+dY7ZtUUNitFT7rOfg1WFQgdT86jLso9ojA86YZ0xzIv1qpYBpAzDgH4mpksiTlwpomtox5L4+BzUgtcclj9atsVUChHp0fVlHwqQWSjgIAP+elX1iA6tnyAp4QYquwdUUBaKGH7c/tUotVAyCfXmrRUdM4+dI8kSfeI4qWGiFY0H4c58zml7tByw4+FI91CBwdxxxQ/UNbt443XIVh5nmgmrSYdXq2kNjuN+pmIn8BYD4Y/mrLnFY7QtSM/aNN/SQMoPlx/wCBWnnnGcA1tcKdGCM7VgLthbG/eKCNSy43uAQM+AHPUcdKp23ZGTYN7RIPLGa00RBlD+NTzSgVdTlHhFHjjJ2wHZ6BaQMe+fvipxtxgA+tWp5UhurS2RVjhGThRgDior68W2R3UgHJJyM5rI6jrRluO+jLRyj2SM5R/D5GrpSl2UbjDoe+qm51BpwctOzMB89qD5Dn51VlvWe4baeAxFC9NkaOJJD95AAPiBiph7AA8TyaeopGdybPUNBvpJtJg7ts92NhOOmOn5YqafUoouJrxFPuhufoKy3ZW3j1BHhllkVUG7arYB8P4rUQabZ2/wD04Ez5kZrj56hkaOzgbnjTKv8AmaynFrbXFwfPbtH505V1WXkR21uPAOS5NEgfwqB8BSSKQuWwBnxNZ3MeoBAzRrwXGfSo3uol67j8qB4kbqT9a4Qk9acLsKtqCg8Ko+LVC+oFjkED0Bqn3SjrWd7QdrNP0WVId8byscHLcDwoN0XhBzfBqGui7E5JJ8ao3+s21iQJ5ApPQZoJqutyRWETgqs86bwi87F8Caxj3F1ezs4s7mXP+o3GfrzVYuc+kMcMeP8Atmzv+1kJXFqpY+dZLULq8vL9JlLdcbR41PZ2N1Ifattg/wBz/wDitBpejX0colhTafBtnT5misai7YXnTVRL2g6VIgjurxO7dfuKeDRh4z7PmRmqsGh3LSpNdXRYqQ23dnpROZfbX0QfpWnBJc0zn+Qm3bRXUlBQ/UdR+zsA2eTiiI5iJ9aEazbJJG27PTIIPStS7MsuuDN63qLzzNGuQo60CuCdjcZyPOrl7/VUyL99eG9aGSyEqa0JcGaUuSbSf61sqn8DEMfhVwqWYvjGegoRol3suZrckjd7S4/P9qI3NysIP9JnPq3/ALpcs+ODqT5HY/EzZVtCPBqexMhXUzH/AHEI6/P9q3fck9f0rzb/AA+vYm1eR7rZGkcRZTk9cgfua9AF3c3fFhb7U/vSjA+Qrl+VNZJ7R6Opgxyww1n2WikcKFnYIo8ScUPu547+PureKeZVbJeM7R9T161Zi0xHYSXkrXL+TfdHwFEViCgAAKB0FZlS65G8vsEshQZlZIx/uYCqVxqmnW/D3W9vdjGaBR6Lqd4d04cD3pn/AGoha9mIY8faJt3mFH807aC+bF1N/wCCv2hhJxa2pY+bmqkLyTz4XT7fbISXVIl9r1PnR+DTrOAf07cMR4vzVkcY9kKB4L4UHlVUkWjFp22Zqy7O3kheW8dTNIcs7noPAAeAAopb9n7ZOZnaQ+Q4FEe8GcDnnk+VOYnOCx+VV9k6qwuEW9muSOO3tLUf0oUU+eMn61KXkb7qkfGkHGCMbs9TSLudjtz16CqBJBtUe2dx9OlRXPszN5bQKkEGeuAegqrfvtc8+Na/F5bM3kcJFZ3EdrIT+Fsms3rt9xtjOCR1rQT4IlQ9HWsPqgeOXa5JA+6a6MFbOfkdIohvbOfGhl8vdMfdNX286r3QEkZVutPM9Wgdplu0t4XjI3KDyf0+dE2jNzAHUcnzqv2fcQaipdd0cbiRgfEDnFaVhFY6Q93IB3s27YvguT4Vx/PqM0/k9D+Jk5Y2vg7/AAxjjfXZVmUN/QYqCM8grXrIU4HlXlH+GELydo++GdscDlvmQP3r1jNZe+Rub+hOB06+dcMnzpJXjhjaWZ1RF5LMcAVldV7VsJNmngKgP/UZclvl4CrKLYlug1iRs8Y+NNGQQCy5B54zTWlySFO4k8YNMfvHPOzZ4gj96WXolaTaCznaoHjzmoWlTumYqzeh4psUb4LS/eHGAenyzUiRrkhUzz1J6ULIcsjFfYXHjinxljncw4HzqRY26NgDyFSCML4Z55NSyUNXapOeSOualGCOOB6UqqSPQeNVLvVLO04eXe/uoc1ZRcugNpFsKTjJPr60IvyXfI6Z8Kk07UptRvVj2CK3ALEeLCo9RjEUjrjgE1t8aGnZj8iWxVuXCorcdMc1ldTkTvHBTfE3Vc8g+Y8qKajNNFGVblPM9R/NALk9+d27muhAwTBcqMjHYcr4ZqlPIw/CavXbvE21Imahl19pk6gxr5Ba0d/Bl6fZNoUT3OqC3TgzDbny5HP0zWj7XNHFDFbJ0UAAelUOwtiW1OS5ZnIhjJ5PieP5pval+8vwM+0T0rz/AOQlfkJfR6n8VGvG2+za/wCFdl3en3V2VGZHCKfQDJ/WtRq2sWulp/UO+YjiNTz8/IVj7HXG0vQ4NPs0EciL7cx5yTycUDmunuJGYsWJPJJyT8TQjGlyKyT2k6CWr63c6i+6V/ZH3Y1+6P5+NDkOeW5+NQgjIyaSWcIF86t2USo9L7nkYHX14/8AVSLEM8YB9BU4UDyHPlTxk8DOfQVnGkKxDOTjmpFVVHH5V08kNupe6mVAPAnJ+lA7ztTEh7qwjMj9A2MmrrG2Vckg8RtXdIQijnLHFCbzX7K1JSAGeT06UOSx1bV2D3chhibwPU/KjFjotnZgYj3v4s/NG4R/0H7MFg6xqxBOYIT58URsdBtbch5czP1y3T6UUHHI+QpwBLYHSqubZZRSIJIVWUSKuNqbSAPUGgepTOtyWnLpGxBWVBx86Nb2N48SsMogxk4yTUdxaSPkpiNz1VhlH/im4fJ9bqXQrLg3VxMhfSXEYJEglgbo6jgfEUBuEkDEhlOfIVsdQt7aM7bm1MbHIZowdo+a/wAUBv7O1QFra4LDxWTg/LOM11MWfHLpnNy4Mi+AE8Ujj2pCB5Diq8sG0cM5+LUTYJ4MoqbT9ObVbnuIHXgZds/dHrT3khFW2KjhnJ0kyxogbTdClupAA07ez8Bx+uay8Tm81ZppPaVTn+K2nam7tdO0u209EaaQDaMMFwAOpzmsrZWwjiWTBHe+0Aeo5xg1wZxcsryfZ6OGSOPAsa7RZldnUljXKQkdR3LBY8Kec1Xmn2R9eaYk2ZeiWacIM56ChOoal3bADk+XlVa+vwgxuG7Hn0oaqmUl2XJPrTVGhbkfRd7qFjYAmecFh+BDQG67T3Vyxh0yAjPTA5NJYdmZJSJNQm3E/hU/qa0FpZQWiBLeFEU+IHNZ94x/lDdW+zNwaDqF8/ealOUB52Zya0FjpdpYL/QhAYdXbkmrhySR4GuG4/dyT0wDxS3Jy7LJJdHbvT6jpS43kY6U9Y8nP6U/gDFSiWNCDxxT+B5YpM01slSPSj0ADwTb7m5OxXL8hS20nnwND73tCbWRoR3gcfglGCP5qrqd49tA6RlgZBg7T4VkLsyNzvkwOmWzSpK2Nj0aGXXrp8soTvF4ZgecZ6Ulrm8YyTWV1cv5iTOPlisNPcPa3K3DMzgDDKT1FbrQ0jm7uSNElVlBVS+3PwNVouxNSsvs8YdYHjOMlGIJH5UT0ELaaa7jaJHw7t8RkD6Yqlqd+v2mRI9y7TtILMR+tZPtJrM6zW9tFId5kMspXhST0HyUAVV2zRhr5F7Xah32pAx7WVBghlBB/wCfvXQzM8EbynJ2jgDHHwoDI93qdw8jKxHebWIHC/8AMUTnnEQMY6jgVpwxfQnynH4G3dyBxmhV7dlWZM+34jyqG/vBEww2X8vKqaBn9vG8Hr51sSo57dkIjdnLZD555q7CkYX243Q/7c8/Spba3glIHKP5dDRS20+bkRjvOOm3miVSP//Z</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -801,6 +858,9 @@
       <c r="F20">
         <v>2</v>
       </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -821,6 +881,9 @@
       <c r="F21">
         <v>2</v>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -841,6 +904,9 @@
       <c r="F22">
         <v>2</v>
       </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -861,6 +927,9 @@
       <c r="F23">
         <v>2</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -881,6 +950,9 @@
       <c r="F24">
         <v>2</v>
       </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -901,6 +973,9 @@
       <c r="F25">
         <v>2</v>
       </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -921,17 +996,20 @@
       <c r="F26">
         <v>1</v>
       </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -952,6 +1030,9 @@
       <c r="F1" t="str">
         <v>Estado</v>
       </c>
+      <c r="G1" t="str">
+        <v>Foto</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -972,6 +1053,9 @@
       <c r="F2">
         <v>2</v>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -992,6 +1076,9 @@
       <c r="F3">
         <v>2</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -1012,6 +1099,9 @@
       <c r="F4">
         <v>2</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -1032,6 +1122,9 @@
       <c r="F5">
         <v>2</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1052,6 +1145,9 @@
       <c r="F6">
         <v>2</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1072,6 +1168,9 @@
       <c r="F7">
         <v>2</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -1092,6 +1191,9 @@
       <c r="F8">
         <v>2</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -1112,6 +1214,9 @@
       <c r="F9">
         <v>0</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -1132,6 +1237,9 @@
       <c r="F10">
         <v>2</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -1152,6 +1260,9 @@
       <c r="F11">
         <v>2</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -1172,6 +1283,9 @@
       <c r="F12">
         <v>2</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -1192,17 +1306,20 @@
       <c r="F13">
         <v>2</v>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1223,6 +1340,9 @@
       <c r="F1" t="str">
         <v>Estado</v>
       </c>
+      <c r="G1" t="str">
+        <v>Foto</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -1243,6 +1363,9 @@
       <c r="F2">
         <v>2</v>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -1263,6 +1386,9 @@
       <c r="F3">
         <v>2</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -1283,6 +1409,9 @@
       <c r="F4">
         <v>2</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -1303,6 +1432,9 @@
       <c r="F5">
         <v>2</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1323,6 +1455,9 @@
       <c r="F6">
         <v>2</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1343,6 +1478,9 @@
       <c r="F7">
         <v>2</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -1363,6 +1501,9 @@
       <c r="F8">
         <v>2</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -1383,6 +1524,9 @@
       <c r="F9">
         <v>2</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -1403,6 +1547,9 @@
       <c r="F10">
         <v>2</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -1423,6 +1570,9 @@
       <c r="F11">
         <v>0</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -1443,6 +1593,9 @@
       <c r="F12">
         <v>2</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -1463,10 +1616,13 @@
       <c r="F13">
         <v>2</v>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>